<commit_message>
extent report manager script added
</commit_message>
<xml_diff>
--- a/TestData/testdata.xlsx
+++ b/TestData/testdata.xlsx
@@ -47,13 +47,13 @@
     <t>impressive</t>
   </si>
   <si>
-    <t xml:space="preserve"> Bairi Kalyanpur Kanpur Nagar</t>
-  </si>
-  <si>
     <t>value</t>
   </si>
   <si>
     <t>status</t>
+  </si>
+  <si>
+    <t>Bairi Kalyanpur Kanpur Nagar</t>
   </si>
 </sst>
 </file>
@@ -472,7 +472,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -507,10 +507,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>11</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -526,7 +526,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
wt & click actions script
</commit_message>
<xml_diff>
--- a/TestData/testdata.xlsx
+++ b/TestData/testdata.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B97ECF-39B4-4446-A50B-CECFF3791D12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Full Name</t>
   </si>
@@ -54,13 +56,76 @@
   </si>
   <si>
     <t>Bairi Kalyanpur Kanpur Nagar</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Sanjay</t>
+  </si>
+  <si>
+    <t>Vivek</t>
+  </si>
+  <si>
+    <t>Ankit</t>
+  </si>
+  <si>
+    <t>Rohan</t>
+  </si>
+  <si>
+    <t>Aman</t>
+  </si>
+  <si>
+    <t>Ajay</t>
+  </si>
+  <si>
+    <t>Harsh</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>anurag@gmail.com</t>
+  </si>
+  <si>
+    <t>sanjay@gmail.com</t>
+  </si>
+  <si>
+    <t>vivek@gmail.com</t>
+  </si>
+  <si>
+    <t>ankit@gmail.com</t>
+  </si>
+  <si>
+    <t>rohan@gmail.com</t>
+  </si>
+  <si>
+    <t>aman@gmail.com</t>
+  </si>
+  <si>
+    <t>ajay@gmail.com</t>
+  </si>
+  <si>
+    <t>harsh@gmail.com</t>
+  </si>
+  <si>
+    <t>ravi@gmail.com</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>raj@gmail.com</t>
+  </si>
+  <si>
+    <t>Patel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +162,14 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -121,21 +194,19 @@
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -147,14 +218,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -192,7 +266,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -264,7 +338,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -437,59 +511,47 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.81640625" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -497,47 +559,161 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="7" t="b">
+      <c r="B2" s="3" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="7" t="b">
+      <c r="B3" s="3" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7" t="b">
+      <c r="B4" s="3" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ADEC8CB-6163-4DD8-8B6F-FA15D9F0401D}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="20.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{72EDA64C-5534-48C1-BB45-6D0A7FAFD971}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{11F84268-3DB4-4762-802C-FBBFD91E9ADB}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{357803C4-7DB6-4ABE-8148-76FE8B988E67}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{CD2659AD-61B5-409D-A052-7FEE2B9D385B}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{1175EA6C-F71A-4086-B2CD-58EBA3D34D74}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{24C0F838-C677-4847-80B6-5D78FC1716A7}"/>
+    <hyperlink ref="B8" r:id="rId7" xr:uid="{3320227F-22A5-477A-8052-DBD597DFCAAC}"/>
+    <hyperlink ref="B9" r:id="rId8" xr:uid="{B72AE76C-E8BE-4BF9-806B-FC869AD52786}"/>
+    <hyperlink ref="B10" r:id="rId9" xr:uid="{4279BDEB-1DD6-4450-849B-E525CA0612CE}"/>
+    <hyperlink ref="B11" r:id="rId10" xr:uid="{06D1756F-2C40-4836-BD04-F75B71580117}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
alert test script done
</commit_message>
<xml_diff>
--- a/TestData/testdata.xlsx
+++ b/TestData/testdata.xlsx
@@ -4,18 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>Full Name</t>
   </si>
@@ -54,6 +55,66 @@
   </si>
   <si>
     <t>Bairi Kalyanpur Kanpur Nagar</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Ajay</t>
+  </si>
+  <si>
+    <t>Ankit</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Shivam</t>
+  </si>
+  <si>
+    <t>Neeraj</t>
+  </si>
+  <si>
+    <t>Vikas</t>
+  </si>
+  <si>
+    <t>Hari</t>
+  </si>
+  <si>
+    <t>Harsh</t>
+  </si>
+  <si>
+    <t>anurag@gmail.com</t>
+  </si>
+  <si>
+    <t>ajay@gmail.com</t>
+  </si>
+  <si>
+    <t>ankit@gmail.com</t>
+  </si>
+  <si>
+    <t>raj@gmail.com</t>
+  </si>
+  <si>
+    <t>rahul@gmail.com</t>
+  </si>
+  <si>
+    <t>shivam@gmail.com</t>
+  </si>
+  <si>
+    <t>neeraj@gmail.com</t>
+  </si>
+  <si>
+    <t>vikas@gmail.com</t>
+  </si>
+  <si>
+    <t>hari@gmail.com</t>
+  </si>
+  <si>
+    <t>harsh@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -119,7 +180,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -136,6 +197,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -540,4 +602,118 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B3" r:id="rId2"/>
+    <hyperlink ref="B4:B11" r:id="rId3" display="ajay@gmail.com"/>
+    <hyperlink ref="B4" r:id="rId4"/>
+    <hyperlink ref="B5" r:id="rId5"/>
+    <hyperlink ref="B6" r:id="rId6"/>
+    <hyperlink ref="B7" r:id="rId7"/>
+    <hyperlink ref="B8" r:id="rId8"/>
+    <hyperlink ref="B9" r:id="rId9"/>
+    <hyperlink ref="B10" r:id="rId10"/>
+    <hyperlink ref="B11" r:id="rId11"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>